<commit_message>
modified the review file for requirements and made the 2nd version for the requirements doc
</commit_message>
<xml_diff>
--- a/lab1/MyDrinkShop/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/lab1/MyDrinkShop/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">do not print this form</t>
   </si>
@@ -90,6 +90,51 @@
     <t xml:space="preserve">Comments/ improvements</t>
   </si>
   <si>
+    <t>R01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerinte funcționale, pct. 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se specifică faptul că fiecare produs trebuie să aparțină unui tip și unei categorii, dar nu se definește diferența dintre ele =&gt; lipsǎ de claritate</t>
+  </si>
+  <si>
+    <t>R02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerințe funcționale, pct. 1 &amp; 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nu există o specificație clară a atributelor pentru entități. De exemplu: Ce câmpuri are un Produs? (Doar nume, preț? Sau și descriere, volum?). Ce câmpuri are un Ingredient? (Doar nume și cantitate? Și unitatea de măsură - ml, g, buc? Preț?).</t>
+  </si>
+  <si>
+    <t>R04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerințe non-funcționale, pct. 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persistența este în fișiere text, dar nu se specifică starea inițială a sistemului. Cum pornește aplicația prima dată? </t>
+  </si>
+  <si>
+    <t>R06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toate punctele</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se menționează "utilizatorul", dar nu se precizează rolurile. Există un singur tip de utilizator (administrator + casier)? Sau există roluri separate?</t>
+  </si>
+  <si>
+    <t>R07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerințe non-funcționale, pct. 1 &amp; 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se specifică "aplicație desktop Java" cu "JavaFX", dar nu se menționează versiunea minimă de Java sau compatibilitatea. De asemenea, nu se specifică sistemul de operare țintă (Windows, Linux, macOS) sau dacă este cross-platform.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Effort to review document (hours):</t>
   </si>
   <si>
@@ -115,6 +160,16 @@
   </si>
   <si>
     <t xml:space="preserve">Pastin Maria, Pecsar Stefania, Popoviciu Luca</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DrinkShopController.java - linia 182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generarea de ID-uri non-unice prin dimensiunea listei. ID-ul este derivat din numărul curent de rețete, nu dintr-un auto-increment real. Dacă o rețetă este ștearsă, dimensiunea listei scade — iar următorul ID generat va intra în conflict cu unul deja
+   existent, cauzând coruperea silențioasă a datelor. Improvement: max(ID-uri existente) + 1</t>
   </si>
   <si>
     <t xml:space="preserve">Tool-based Code Analysis</t>
@@ -145,7 +200,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -187,6 +242,11 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.500000"/>
+      <color rgb="FF0F1115"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="5">
@@ -285,7 +345,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -320,6 +380,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="5" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="6" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf fontId="5" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -886,7 +949,8 @@
   <cols>
     <col min="1" max="1" style="1" width="8.90625"/>
     <col customWidth="1" min="2" max="2" style="1" width="12.26953125"/>
-    <col customWidth="1" min="3" max="4" style="1" width="16.26953125"/>
+    <col customWidth="1" min="3" max="3" style="1" width="16.26953125"/>
+    <col customWidth="1" min="4" max="4" style="1" width="30.8515625"/>
     <col customWidth="1" min="5" max="5" style="1" width="41.453125"/>
     <col min="6" max="8" style="1" width="8.90625"/>
     <col customWidth="1" min="9" max="9" style="1" width="21"/>
@@ -1000,49 +1064,79 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="57">
       <c r="B10" s="6">
         <v>1</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18"/>
-    </row>
-    <row r="11">
+      <c r="C10" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" ht="99.75">
       <c r="B11" s="6">
         <f t="shared" ref="B11:B25" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
-    </row>
-    <row r="12">
+      <c r="C11" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" ht="42.75">
       <c r="B12" s="6">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="18"/>
-    </row>
-    <row r="13">
+      <c r="C12" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" ht="57">
       <c r="B13" s="6">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="18"/>
-    </row>
-    <row r="14">
+      <c r="C13" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" ht="99.75">
       <c r="B14" s="6">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18"/>
+      <c r="C14" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="6">
@@ -1051,7 +1145,7 @@
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="18"/>
+      <c r="E15" s="19"/>
     </row>
     <row r="16">
       <c r="B16" s="6">
@@ -1060,7 +1154,7 @@
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="18"/>
+      <c r="E16" s="19"/>
     </row>
     <row r="17">
       <c r="B17" s="6">
@@ -1069,7 +1163,7 @@
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="18"/>
+      <c r="E17" s="19"/>
     </row>
     <row r="18">
       <c r="B18" s="6">
@@ -1078,7 +1172,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
-      <c r="E18" s="19"/>
+      <c r="E18" s="20"/>
     </row>
     <row r="19">
       <c r="B19" s="6">
@@ -1087,7 +1181,7 @@
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="19"/>
+      <c r="E19" s="20"/>
     </row>
     <row r="20">
       <c r="B20" s="6">
@@ -1096,7 +1190,7 @@
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="19"/>
+      <c r="E20" s="20"/>
     </row>
     <row r="21">
       <c r="B21" s="6">
@@ -1105,7 +1199,7 @@
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
-      <c r="E21" s="19"/>
+      <c r="E21" s="20"/>
     </row>
     <row r="22">
       <c r="B22" s="6">
@@ -1114,7 +1208,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="19"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23">
       <c r="B23" s="6">
@@ -1123,7 +1217,7 @@
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
-      <c r="E23" s="19"/>
+      <c r="E23" s="20"/>
     </row>
     <row r="24">
       <c r="B24" s="6">
@@ -1132,7 +1226,7 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
-      <c r="E24" s="19"/>
+      <c r="E24" s="20"/>
     </row>
     <row r="25">
       <c r="B25" s="6">
@@ -1141,14 +1235,16 @@
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
-      <c r="E25" s="19"/>
+      <c r="E25" s="20"/>
     </row>
     <row r="27">
-      <c r="C27" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="17"/>
+      <c r="C27" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="22"/>
+      <c r="E27" s="17">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1197,7 +1293,7 @@
     </row>
     <row r="2">
       <c r="B2" s="5" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1222,13 +1318,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="23"/>
+      <c r="D4" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="24"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1240,13 +1336,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="25"/>
+      <c r="C5" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="26"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1295,8 +1391,8 @@
         <v>1</v>
       </c>
       <c r="C10" s="17"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
     </row>
     <row r="11">
       <c r="B11" s="6">
@@ -1304,8 +1400,8 @@
         <v>2</v>
       </c>
       <c r="C11" s="17"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
     </row>
     <row r="12">
       <c r="B12" s="6">
@@ -1314,7 +1410,7 @@
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="18"/>
+      <c r="E12" s="19"/>
     </row>
     <row r="13">
       <c r="B13" s="6">
@@ -1323,7 +1419,7 @@
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="18"/>
+      <c r="E13" s="19"/>
     </row>
     <row r="14">
       <c r="B14" s="6">
@@ -1331,8 +1427,8 @@
         <v>5</v>
       </c>
       <c r="C14" s="17"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
     </row>
     <row r="15">
       <c r="B15" s="6">
@@ -1341,7 +1437,7 @@
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="18"/>
+      <c r="E15" s="19"/>
     </row>
     <row r="16">
       <c r="B16" s="6">
@@ -1349,8 +1445,8 @@
         <v>7</v>
       </c>
       <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
     </row>
     <row r="17">
       <c r="B17" s="6">
@@ -1358,8 +1454,8 @@
         <v>8</v>
       </c>
       <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
     </row>
     <row r="18">
       <c r="B18" s="6">
@@ -1368,7 +1464,7 @@
       </c>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="18"/>
+      <c r="E18" s="19"/>
     </row>
     <row r="19">
       <c r="B19" s="6">
@@ -1376,8 +1472,8 @@
         <v>10</v>
       </c>
       <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
     </row>
     <row r="20">
       <c r="B20" s="6">
@@ -1386,7 +1482,7 @@
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="18"/>
+      <c r="E20" s="19"/>
     </row>
     <row r="21">
       <c r="B21" s="6">
@@ -1395,7 +1491,7 @@
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="18"/>
+      <c r="E21" s="19"/>
     </row>
     <row r="22">
       <c r="B22" s="6">
@@ -1404,7 +1500,7 @@
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="18"/>
+      <c r="E22" s="19"/>
     </row>
     <row r="23">
       <c r="B23" s="6">
@@ -1413,7 +1509,7 @@
       </c>
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="18"/>
+      <c r="E23" s="19"/>
     </row>
     <row r="24">
       <c r="B24" s="6">
@@ -1422,7 +1518,7 @@
       </c>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="18"/>
+      <c r="E24" s="19"/>
     </row>
     <row r="25">
       <c r="B25" s="6">
@@ -1431,7 +1527,7 @@
       </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="18"/>
+      <c r="E25" s="19"/>
     </row>
     <row r="26">
       <c r="B26" s="6">
@@ -1440,13 +1536,13 @@
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="18"/>
+      <c r="E26" s="19"/>
     </row>
     <row r="28">
-      <c r="C28" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D28" s="21"/>
+      <c r="C28" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="22"/>
       <c r="E28" s="17"/>
     </row>
   </sheetData>
@@ -1497,7 +1593,7 @@
     </row>
     <row r="2">
       <c r="B2" s="5" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1522,13 +1618,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="27"/>
+      <c r="D4" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="28"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1540,13 +1636,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" s="26" t="s">
+      <c r="C5" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="29"/>
+      <c r="D5" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="30"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1563,7 +1659,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="E6" s="14"/>
     </row>
@@ -1594,9 +1690,15 @@
       <c r="B10" s="6">
         <v>1</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
+      <c r="C10" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="6">
@@ -1605,7 +1707,7 @@
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
+      <c r="E11" s="19"/>
     </row>
     <row r="12">
       <c r="B12" s="6">
@@ -1614,7 +1716,7 @@
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="18"/>
+      <c r="E12" s="19"/>
     </row>
     <row r="13">
       <c r="B13" s="6">
@@ -1622,8 +1724,8 @@
         <v>4</v>
       </c>
       <c r="C13" s="17"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
     </row>
     <row r="14">
       <c r="B14" s="6">
@@ -1631,8 +1733,8 @@
         <v>5</v>
       </c>
       <c r="C14" s="17"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
     </row>
     <row r="15">
       <c r="B15" s="6">
@@ -1640,8 +1742,8 @@
         <v>6</v>
       </c>
       <c r="C15" s="17"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
     </row>
     <row r="16">
       <c r="B16" s="6">
@@ -1649,8 +1751,8 @@
         <v>7</v>
       </c>
       <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
     </row>
     <row r="17">
       <c r="B17" s="6">
@@ -1658,8 +1760,8 @@
         <v>8</v>
       </c>
       <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
     </row>
     <row r="18">
       <c r="B18" s="6">
@@ -1667,8 +1769,8 @@
         <v>9</v>
       </c>
       <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
     </row>
     <row r="19">
       <c r="B19" s="6">
@@ -1677,7 +1779,7 @@
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="18"/>
+      <c r="E19" s="19"/>
     </row>
     <row r="20">
       <c r="B20" s="6">
@@ -1685,8 +1787,8 @@
         <v>11</v>
       </c>
       <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
     </row>
     <row r="21">
       <c r="B21" s="6">
@@ -1695,7 +1797,7 @@
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="18"/>
+      <c r="E21" s="19"/>
     </row>
     <row r="22">
       <c r="B22" s="6">
@@ -1703,8 +1805,8 @@
         <v>13</v>
       </c>
       <c r="C22" s="17"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
     </row>
     <row r="23">
       <c r="B23" s="6">
@@ -1712,8 +1814,8 @@
         <v>14</v>
       </c>
       <c r="C23" s="17"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
     </row>
     <row r="24">
       <c r="B24" s="6">
@@ -1721,8 +1823,8 @@
         <v>15</v>
       </c>
       <c r="C24" s="17"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
     </row>
     <row r="25">
       <c r="B25" s="6">
@@ -1730,8 +1832,8 @@
         <v>16</v>
       </c>
       <c r="C25" s="17"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
     </row>
     <row r="26">
       <c r="B26" s="6">
@@ -1740,7 +1842,7 @@
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="18"/>
+      <c r="E26" s="19"/>
     </row>
     <row r="27">
       <c r="B27" s="6">
@@ -1748,7 +1850,7 @@
         <v>18</v>
       </c>
       <c r="C27" s="17"/>
-      <c r="D27" s="18"/>
+      <c r="D27" s="19"/>
       <c r="E27" s="17"/>
     </row>
     <row r="28">
@@ -1757,8 +1859,8 @@
         <v>19</v>
       </c>
       <c r="C28" s="17"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
     </row>
     <row r="29">
       <c r="B29" s="6">
@@ -1766,8 +1868,8 @@
         <v>20</v>
       </c>
       <c r="C29" s="17"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
     </row>
     <row r="30">
       <c r="B30" s="6">
@@ -1775,14 +1877,14 @@
         <v>21</v>
       </c>
       <c r="C30" s="17"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
     </row>
     <row r="32">
-      <c r="C32" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D32" s="21"/>
+      <c r="C32" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="22"/>
       <c r="E32" s="17"/>
     </row>
   </sheetData>
@@ -1834,7 +1936,7 @@
     </row>
     <row r="2">
       <c r="B2" s="5" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1859,13 +1961,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="27"/>
+      <c r="C4" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="28"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1910,16 +2012,16 @@
         <v>19</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10">
@@ -1927,9 +2029,9 @@
         <v>1</v>
       </c>
       <c r="C10" s="17"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
     </row>
     <row r="11">
       <c r="B11" s="6">
@@ -1938,8 +2040,8 @@
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
     </row>
     <row r="12">
       <c r="B12" s="6">
@@ -1948,8 +2050,8 @@
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
     </row>
     <row r="13">
       <c r="B13" s="6">
@@ -1957,9 +2059,9 @@
         <v>4</v>
       </c>
       <c r="C13" s="17"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
     </row>
     <row r="14">
       <c r="B14" s="6">
@@ -1967,9 +2069,9 @@
         <v>5</v>
       </c>
       <c r="C14" s="17"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
     </row>
     <row r="15">
       <c r="B15" s="6">
@@ -1977,9 +2079,9 @@
         <v>6</v>
       </c>
       <c r="C15" s="17"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
     </row>
     <row r="16">
       <c r="B16" s="6">
@@ -1987,9 +2089,9 @@
         <v>7</v>
       </c>
       <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
     </row>
     <row r="17">
       <c r="B17" s="6">
@@ -1997,9 +2099,9 @@
         <v>8</v>
       </c>
       <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
     </row>
     <row r="18">
       <c r="B18" s="6">
@@ -2007,9 +2109,9 @@
         <v>9</v>
       </c>
       <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
     </row>
     <row r="19">
       <c r="B19" s="6">
@@ -2018,8 +2120,8 @@
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
     </row>
     <row r="20">
       <c r="B20" s="6">
@@ -2027,9 +2129,9 @@
         <v>11</v>
       </c>
       <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
     </row>
     <row r="21">
       <c r="B21" s="6">
@@ -2038,8 +2140,8 @@
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
     </row>
     <row r="22">
       <c r="B22" s="6">
@@ -2047,9 +2149,9 @@
         <v>13</v>
       </c>
       <c r="C22" s="17"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
     </row>
     <row r="23">
       <c r="B23" s="6">
@@ -2057,9 +2159,9 @@
         <v>14</v>
       </c>
       <c r="C23" s="17"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
     </row>
     <row r="24">
       <c r="B24" s="6">
@@ -2067,9 +2169,9 @@
         <v>15</v>
       </c>
       <c r="C24" s="17"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
     </row>
     <row r="25">
       <c r="B25" s="6">
@@ -2077,9 +2179,9 @@
         <v>16</v>
       </c>
       <c r="C25" s="17"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
     </row>
     <row r="26">
       <c r="B26" s="6">
@@ -2088,8 +2190,8 @@
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
     </row>
     <row r="27">
       <c r="B27" s="6">
@@ -2097,7 +2199,7 @@
         <v>18</v>
       </c>
       <c r="C27" s="17"/>
-      <c r="D27" s="18"/>
+      <c r="D27" s="19"/>
       <c r="E27" s="17"/>
       <c r="F27" s="17"/>
     </row>
@@ -2107,9 +2209,9 @@
         <v>19</v>
       </c>
       <c r="C28" s="17"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
     </row>
     <row r="29">
       <c r="B29" s="6">
@@ -2117,9 +2219,9 @@
         <v>20</v>
       </c>
       <c r="C29" s="17"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
     </row>
     <row r="30">
       <c r="B30" s="6">
@@ -2127,17 +2229,17 @@
         <v>21</v>
       </c>
       <c r="C30" s="17"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
     </row>
     <row r="32">
-      <c r="C32" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="32"/>
+      <c r="C32" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="33"/>
     </row>
     <row r="35">
       <c r="F35" s="1"/>

</xml_diff>